<commit_message>
Update: Threat Alert Report - 2026-05-29 15:49
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_HMB_threats.xlsx
+++ b/excel_routes/route_AHB_HMB_threats.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -532,7 +532,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>24-MAY-26</t>
+          <t>12-JUL-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -546,13 +546,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>971</v>
+        <v>1101</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1312</v>
+        <v>1368</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-341</v>
+        <v>-267</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -591,13 +591,13 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>671</v>
+        <v>763</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1221</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-550</v>
+        <v>-458</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -614,6 +614,96 @@
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>19-JUL-26</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SM-446</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-346</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>915</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1221</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>-306</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>19-JUL-26</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SM-446</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>flyadeal F3-342</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>985</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1221</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>-236</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>SAR</t>
         </is>

</xml_diff>